<commit_message>
analytics: multi-period trends, forecasts, 12 correlations, enhanced confidence, anomaly filter
- indicators.py: +4 functions (multi_period_trend, price_forecast, change_from_baseline, enhanced_confidence)
- precompute_analysis.py: 4→12 correlation pairs, multi-period table, forecast display, '3 Hal Penting', anomaly filter
- create_excel.py: fix path ~/sembako/ → ~/sembako/data/
- fetch_cuaca_pagi.py: fix path ~/sembako/ → ~/sembako/data/
- update_crypto.py: fix HISTORY_PATH to data/
- update_emas.py: fix HISTORY_PATH to data/
- cuaca_yogyakarta.xlsx: synced from root to data/
- harga_sembako.xlsx: synced cache data to 30 Jun
</commit_message>
<xml_diff>
--- a/data/cuaca_yogyakarta.xlsx
+++ b/data/cuaca_yogyakarta.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,23 +486,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22.9</v>
+        <v>25.7</v>
       </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>29.9</v>
       </c>
       <c r="E2" t="n">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>5.7</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -513,14 +513,152 @@
         <v>30.2</v>
       </c>
       <c r="J2" t="n">
-        <v>22.9</v>
+        <v>23.5</v>
       </c>
       <c r="K2" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>Gerimis Sedang</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>20:28</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>82</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Mendung</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="J3" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Gerimis Sedang</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>07:01</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>94</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Cerah Sebagian</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Gerimis Ringan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>13:43</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>52</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Mendung</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Gerimis Ringan</t>
         </is>
       </c>
     </row>

</xml_diff>